<commit_message>
chore(marketing): update creator kit and UGC ops sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/CortiFree_Creator_Kit.xlsx
+++ b/marketing/CortiFree_Creator_Kit.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Hook bank" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 App screens to film" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Before you post" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 New features" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -606,7 +607,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>An app to stress less and lower your cortisol, with an AI companion called Milo. A 2-minute quiz builds your 66-day plan; Milo checks in with you every day and picks the right breathing, meditation or sleep story for the moment. You can give Milo your iPhone anxiety test result or your ChatGPT conversations, and it gets to know you instantly.</t>
+          <t>An app to stress less and lower your cortisol, with an AI companion called Milo. A 2-minute quiz builds your 28-day plan; Milo checks in with you every day and picks the right breathing, meditation or sleep story for the moment. You can give Milo your iPhone anxiety test result or your ChatGPT conversations, and it gets to know you instantly.</t>
         </is>
       </c>
     </row>
@@ -712,6 +713,625 @@
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>• Check Drive › 05_Winners every Monday.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="006C4CF1"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Sub-promise</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>On-screen hook</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Opening line (first 2s)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Beats (say it YOUR way)</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>APP SHOWCASE (must be on screen)</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Emotional beat</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>CTA</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Caption</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Notes / variants</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Heart rate drop</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Lower stress</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>V1 Snap reaction</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>watch my heart rate drop in 60 seconds</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>My heart is at 96 right now. Give me 60 seconds.</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>1. Home &gt; Calm check: fingertip on the back camera, the heart beats on screen, show the number.
+2. Milo picks the reset (physiological sigh). Do it on camera.
+3. Measure again. Hold the phone to the camera: the new number.
+4. React to the before → after screen.</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>Calm check: live heart + BPM → 60 s reset → before/after screen</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>The moment the second number appears.</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>'Try it, it's in the app.'</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>30–45s</t>
+        </is>
+      </c>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>60 seconds 😮‍💨 #ad #nervoussystem #heartrate #stressrelief</t>
+        </is>
+      </c>
+      <c r="N2" s="15" t="inlineStr">
+        <is>
+          <t>Only your real numbers. Variants: before a meeting / after a fight / at 2am</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Heart rate drop</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Lower stress</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>V7 Duo reaction</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>made my boyfriend do the 60-second heart rate test</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>He says he's chill. His heart says 104.</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>1. Partner measures, you react to the number.
+2. You guide him through the 60 s reset (he's skeptical).
+3. Second measure: both react to the drop.</t>
+        </is>
+      </c>
+      <c r="I3" s="15" t="inlineStr">
+        <is>
+          <t>Calm check before/after screen</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="inlineStr">
+        <is>
+          <t>His face when the number drops.</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>'Tag the one who says he's chill.'</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>30–45s</t>
+        </is>
+      </c>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>he said he was chill 🙂 #ad #couples #heartrate</t>
+        </is>
+      </c>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>Variants: mom, roommate, boss (with permission)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Nervous system reset</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Less anxiety</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>V5 GRWM</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>nervous system reset tricks that actually work (I tested 4)</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>I tried the four nervous system tricks everyone posts. Here's the one that worked for me.</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>1. Show the 60 s reset screen with the 4 techniques.
+2. 10 seconds of each: physiological sigh, humming, butterfly hug, 5-4-3-2-1.
+3. Your honest ranking + the one Milo picks for you.</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>60-second reset: mode picker + each animation</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>'The humming one made me cry a little, not gonna lie.'</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>'Which one are you trying tonight?'</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>40–60s</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>nervous system reset ranking #ad #nervoussystemregulation #vagusnerve</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>Never promise it treats anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Breathe before TikTok</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Lower stress</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>V1 Snap reaction</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>I made TikTok force me to breathe before opening it</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Every time I open TikTok now, this happens.</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>1. Open TikTok on camera: CortiFree pops up instead, 30 s breathing.
+2. 'Still want to scroll?' → you hesitate → 'No, I'm good'.
+3. Quick 3-step setup shown from the guide (Shortcuts &gt; Automation).</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Breathe pause screen + setup guide</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>Laughing at yourself: 'I got played by my own phone.'</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>'Setup is in the app, takes 1 minute.'</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>20–35s</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>my screen time is crying #ad #screentime #iphonehack #dopaminedetox</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>Variant: Instagram, 'girl who can't stop scrolling'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Breathe before TikTok</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Lower stress</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>V3 Green screen</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>iPhone hack to stop doomscrolling (no app blocker)</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>This iPhone hack cut my scrolling and it's not a blocker.</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>1. Green screen: the 5 setup steps.
+2. Show the pause screen.
+3. 'After a pause TikTok opens normally for 10 min, so it never loops.'</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>Setup guide + pause screen</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>'It doesn't block me. It just asks me if I'm okay.'</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>'Save this.'</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>25–35s</t>
+        </is>
+      </c>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>save this iPhone hack #ad #iphonetips #doomscrolling</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Apple Watch body stress</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Lower cortisol</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>V6 Mirror close-up</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>my Apple Watch knew I was stressed before I did</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>(Morning, in bed) I felt fine. My body didn't.</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>1. Open CortiFree: 'Body stress this morning: Under strain', HRV below usual, short night.
+2. 'That explains the jaw.'
+3. Milo adapts the day: gentle plan, 60 s reset now.</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Home body stress card + Milo</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>'I thought I was fine. I wasn't.'</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>'Connect your Watch, it's free in the app.'</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>20–30s</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>my watch called me out #ad #applewatch #hrv #stress</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>Wellness estimate, never 'my cortisol is X'</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>N7</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Decode this message</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Stop ruminating</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>V1 Snap reaction</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>I sent my boss's text to an AI and it calmed me down</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>My boss texted 'can we talk tomorrow?' and I haven't slept.</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>1. Screenshot → Milo → 'Decode this message'.
+2. 'Milo is reading between the lines…'.
+3. Read the tone + meaning + calm reply out loud.
+4. Copy the reply, send it.</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>Decode: screenshot → reading animation → tone, meaning, calm reply</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>Relief: 'okay… I can breathe.'</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>'Next time, send it to Milo before spiraling.'</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>25–40s</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>overthinking a 4-word text #ad #overthinking #anxiety</t>
+        </is>
+      </c>
+      <c r="N8" s="15" t="inlineStr">
+        <is>
+          <t>Variants: crush 'ok.', mom, group chat. Never show someone else's name/number</t>
         </is>
       </c>
     </row>
@@ -848,7 +1468,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>cortisol • cortisol face • stress belly • nervous system • overthinking • 3am • mental load • the strong friend • high-functioning anxiety • burnout • 'I'm fine' • my therapist • Milo • 66 days</t>
+          <t>cortisol • cortisol face • stress belly • nervous system • overthinking • 3am • mental load • the strong friend • high-functioning anxiety • burnout • 'I'm fine' • my therapist • Milo • 28 days</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1691,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Cortisol quiz → result → Milo → 66-day plan · 'Lower your cortisol' session · morning coherence breathing</t>
+          <t>Cortisol quiz → result → Milo → 28-day plan · 'Lower your cortisol' session · morning coherence breathing</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -1338,7 +1958,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -1353,21 +1973,21 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Series + honesty: 'Day 1 of 66', real anxiety score at day 14, real update at day 30.</t>
+          <t>Series + honesty: 'Day 1 of 28', real anxiety score at day 14, real update at day 28, then cycle 2.</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Plan tab Day X/66 · streak · anxiety check result · Milo daily message · 'Why 66 days?'</t>
+          <t>Plan tab (day of the 28-day plan) · streak · anxiety check result · Milo daily message · new cycle</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>• Day 1/66 of lowering my cortisol
+          <t>• Day 1/28 of lowering my cortisol
 • Day 14: I retook my anxiety test
-• Day 30/66: what actually changed
-• it doesn't take 21 days to build a habit
-• what 66 days of this did to my stress</t>
+• Day 28: what actually changed
+• Week 2 of my plan: the day I almost quit
+• why I'm starting a second 28 days</t>
         </is>
       </c>
     </row>
@@ -1515,7 +2135,7 @@
           <t>1. 2–3 seconds of close-ups: puffy eyes, jawline, under-eyes. No filter.
 2. 'Then I learned cortisol, the stress hormone, can do this.' 3 habits in 1 line each: 5h sleep, coffee before water, scrolling in bed.
 3. Open CortiFree: 'Let's check if your cortisol is higher than you think' → answer 3 questions → result.
-4. 'View my 66-day plan' → Milo's first message.</t>
+4. 'View my 28-day plan' → Milo's first message.</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -2550,7 +3170,7 @@
         <is>
           <t>1. Green screen: ChatGPT's generic answer ('try deep breathing, exercise…').
 2. Paste the same chat into Milo → summary personal to you + first step + exercise card you can start.
-3. Show the 66-day plan.</t>
+3. Show the 28-day plan.</t>
         </is>
       </c>
       <c r="I16" s="9" t="inlineStr">
@@ -4022,7 +4642,7 @@
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -4037,22 +4657,22 @@
       </c>
       <c r="E37" s="14" t="inlineStr">
         <is>
-          <t>V8 Day X/66 series</t>
+          <t>V8 Day X/28 series</t>
         </is>
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Day 1/66 of lowering my cortisol</t>
+          <t>Day 1/28 of lowering my cortisol</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>Day 1 of 66 of lowering my cortisol. Let's see if I make it.</t>
+          <t>Day 1 of 28 of lowering my cortisol. Let's see if I make it.</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>1. Show 'Day 1/66' and today's tasks.
+          <t>1. Show 'Day 1' in the Plan tab and today's steps.
 2. Do one on camera (breathing).
 3. Ask Milo one thing, show answer.
 4. Honest 1-line feeling. 'See you on Day 2.'</t>
@@ -4060,7 +4680,7 @@
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>Plan tab + task + Milo</t>
+          <t>Plan tab + step + Milo</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
@@ -4080,12 +4700,12 @@
       </c>
       <c r="M37" s="14" t="inlineStr">
         <is>
-          <t>day 1/66 #ad #66days #cortisol #healingjourney</t>
+          <t>day 1/28 #ad #28daychallenge #cortisol #healingjourney</t>
         </is>
       </c>
       <c r="N37" s="14" t="inlineStr">
         <is>
-          <t>Post Day 1, 2, 3, 7, 14, 21, 30, 45, 66. Same framing every time.</t>
+          <t>Post Day 1, 2, 3, 7, 14, 21, 28. Same framing every time.</t>
         </is>
       </c>
     </row>
@@ -4097,7 +4717,7 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -4112,7 +4732,7 @@
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>V8 Day X/66 series</t>
+          <t>V8 Day X/28 series</t>
         </is>
       </c>
       <c r="F38" s="14" t="inlineStr">
@@ -4128,7 +4748,7 @@
       <c r="H38" s="14" t="inlineStr">
         <is>
           <t>1. First result (real, can blur).
-2. Retake the anxiety check in the Plan tab.
+2. Retake the anxiety check in the Plan tab (it comes back every 2 weeks).
 3. New result → honest reaction, whatever it is.
 4. Milo's comment on it.</t>
         </is>
@@ -4145,7 +4765,7 @@
       </c>
       <c r="K38" s="14" t="inlineStr">
         <is>
-          <t>'Day 30 coming.'</t>
+          <t>'Day 28 coming.'</t>
         </is>
       </c>
       <c r="L38" s="14" t="inlineStr">
@@ -4172,7 +4792,7 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -4182,57 +4802,62 @@
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E39" s="14" t="inlineStr">
         <is>
-          <t>V8 Day X/66 series</t>
+          <t>V8 Day X/28 series</t>
         </is>
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>Day 30/66: what actually changed</t>
+          <t>Day 28: what actually changed</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>Day 30. Here's what actually changed. Honestly.</t>
+          <t>Day 28. Plan finished. Here's what actually changed. Honestly.</t>
         </is>
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>1. 3 real changes, 1 thing that didn't.
-2. Streak + badge.
-3. Milo: 'what should I focus on next?'</t>
+          <t>1. Day 1 clip vs now.
+2. Anxiety check day 1 vs day 28 (real).
+3. 3 real changes, 1 thing that didn't.
+4. Milo's message + 'starting cycle 2'.</t>
         </is>
       </c>
       <c r="I39" s="14" t="inlineStr">
         <is>
-          <t>Streak, badges, Milo</t>
+          <t>Day 1 clip + anxiety check results + Milo + new cycle</t>
         </is>
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>'The thing I didn't expect…'</t>
+          <t>The Day 1 clip: let it play.</t>
         </is>
       </c>
       <c r="K39" s="14" t="inlineStr">
         <is>
-          <t>'Follow for day 66.'</t>
+          <t>'Start your Day 1.'</t>
         </is>
       </c>
       <c r="L39" s="14" t="inlineStr">
         <is>
-          <t>30–45s</t>
+          <t>40–60s</t>
         </is>
       </c>
       <c r="M39" s="14" t="inlineStr">
         <is>
-          <t>halfway #ad #66days #progress</t>
-        </is>
-      </c>
-      <c r="N39" s="14" t="inlineStr"/>
+          <t>28 days later #ad #28daychallenge #progress</t>
+        </is>
+      </c>
+      <c r="N39" s="14" t="inlineStr">
+        <is>
+          <t>Only after 28 real days.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
@@ -4242,7 +4867,7 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
@@ -4257,49 +4882,50 @@
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>V3 Green screen</t>
+          <t>V8 Day X/28 series</t>
         </is>
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
-          <t>it doesn't take 21 days to build a habit</t>
+          <t>Week 2 of my plan: the day I almost quit</t>
         </is>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>'21 days to build a habit' is a myth.</t>
+          <t>Day 9. I almost skipped today. Here's why I didn't.</t>
         </is>
       </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>1. Green screen: UCL research (Lally) — 66 days on average.
-2. 'That's why you quit after 2 weeks.'
-3. Show your 66-day plan + 'Why 66 days?' screen.</t>
+          <t>1. Honest: tired, busy, no motivation.
+2. Milo's message that day (show it).
+3. The 5-minute version you did instead.
+4. Streak still alive.</t>
         </is>
       </c>
       <c r="I40" s="14" t="inlineStr">
         <is>
-          <t>Plan + 'Why 66 days?'</t>
+          <t>Milo message + short session + streak</t>
         </is>
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>'It wasn't you. The timeline was wrong.'</t>
+          <t>'Five minutes counts.'</t>
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr">
         <is>
-          <t>'Start your 66 days.'</t>
+          <t>'Tell me your day count.'</t>
         </is>
       </c>
       <c r="L40" s="14" t="inlineStr">
         <is>
-          <t>20–30s</t>
+          <t>25–35s</t>
         </is>
       </c>
       <c r="M40" s="14" t="inlineStr">
         <is>
-          <t>the 21 days thing was a lie #ad #habits #science</t>
+          <t>showing up when I don't want to #ad #consistency #selfcare</t>
         </is>
       </c>
       <c r="N40" s="14" t="inlineStr"/>
@@ -4312,7 +4938,7 @@
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -4327,57 +4953,52 @@
       </c>
       <c r="E41" s="14" t="inlineStr">
         <is>
-          <t>V8 Day X/66 series</t>
+          <t>V8 Day X/28 series</t>
         </is>
       </c>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>what 66 days of this did to my stress</t>
+          <t>why I'm starting a second 28 days</t>
         </is>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>Sixty-six days ago I couldn't sleep, couldn't relax, couldn't stop.</t>
+          <t>I finished my 28 days. I'm starting again. Here's why.</t>
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>1. Day 1 clip vs now.
-2. Anxiety check day 1 vs day 66 (real).
-3. Milo's final message.
-4. 'Starting cycle 2.'</t>
+          <t>1. What the first cycle changed (real).
+2. What you want next (sleep? focus?).
+3. Change goal in the Plan tab, Milo builds cycle 2.</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr">
         <is>
-          <t>Day 1 clip + anxiety check results + Milo</t>
+          <t>Plan tab: new cycle / change goal + Milo</t>
         </is>
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>The day 1 clip: let it play.</t>
+          <t>'I didn't want to lose this feeling.'</t>
         </is>
       </c>
       <c r="K41" s="14" t="inlineStr">
         <is>
-          <t>'Start your day 1.'</t>
+          <t>'Day 1 again, come with me.'</t>
         </is>
       </c>
       <c r="L41" s="14" t="inlineStr">
         <is>
-          <t>40–60s</t>
+          <t>25–40s</t>
         </is>
       </c>
       <c r="M41" s="14" t="inlineStr">
         <is>
-          <t>66 days later #ad #66days #transformation</t>
-        </is>
-      </c>
-      <c r="N41" s="14" t="inlineStr">
-        <is>
-          <t>Only after 66 real days.</t>
-        </is>
-      </c>
+          <t>cycle 2 #ad #28daychallenge #healingjourney</t>
+        </is>
+      </c>
+      <c r="N41" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4543,7 +5164,7 @@
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Day X/66 series</t>
+          <t>Day X/28 series</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
@@ -5226,12 +5847,12 @@
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>Day 1/66 of lowering my cortisol</t>
+          <t>Day 1/28 of lowering my cortisol</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5869,7 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
     </row>
@@ -5260,12 +5881,12 @@
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>Day 30/66: what actually changed</t>
+          <t>Day 28: what actually changed</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
     </row>
@@ -5277,12 +5898,12 @@
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>it doesn't take 21 days to build a habit</t>
+          <t>Week 2 of my plan: the day I almost quit</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
     </row>
@@ -5294,12 +5915,12 @@
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>what 66 days of this did to my stress</t>
+          <t>why I'm starting a second 28 days</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>66 days, documented</t>
+          <t>28 days, documented</t>
         </is>
       </c>
     </row>
@@ -5501,7 +6122,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Analysis → 'View my 66-day plan' → Plan tab (Day X/66, today's steps)</t>
+          <t>Analysis → 'View my 28-day plan' → Plan tab (day of the 28-day plan, today's steps)</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
@@ -5705,7 +6326,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Streak, badges, 'Why 66 days?'</t>
+          <t>Streak, badges, end of cycle / new cycle</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">

</xml_diff>